<commit_message>
cambios modulo de aulas
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/excel/formatoSeccionesSinAula.xlsx
+++ b/src/main/resources/templates/excel/formatoSeccionesSinAula.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bastards\Documents\NetBeansProjects\lamolina-pivot\src\main\resources\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D05ED67-CD77-4368-A6EC-7F6240E7443E}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{809F9F7D-C635-4924-9B23-D313F057F4B2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -440,9 +440,9 @@
     <col min="2" max="2" width="73.6640625" customWidth="1"/>
     <col min="3" max="3" width="65.109375" customWidth="1"/>
     <col min="4" max="4" width="13.5546875" customWidth="1"/>
-    <col min="5" max="5" width="24.44140625" customWidth="1"/>
-    <col min="6" max="6" width="19.109375" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="30.33203125" customWidth="1"/>
     <col min="8" max="8" width="13.5546875" customWidth="1"/>
     <col min="9" max="9" width="21.44140625" customWidth="1"/>
     <col min="10" max="10" width="11.5546875" customWidth="1"/>
@@ -466,13 +466,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>6</v>

</xml_diff>